<commit_message>
CORTES DE LA SEMANA
</commit_message>
<xml_diff>
--- a/Cosas que llegan de mercado/2026/Periodo 1/Nota7.xlsx
+++ b/Cosas que llegan de mercado/2026/Periodo 1/Nota7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Documents\GitHub\Motozom\Cosas que llegan de mercado\2026\Periodo 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F9102F9-D6C3-4473-9EFB-D6282890BC19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{444D867F-6CFE-4A11-B099-C42BAED0C63B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>Cantidad</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>HAN LLEGADO 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LLEGARON 2 AZULES </t>
   </si>
 </sst>
 </file>
@@ -1123,6 +1126,9 @@
       <c r="J66" t="s">
         <v>5</v>
       </c>
+      <c r="M66" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="67" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J67" t="s">

</xml_diff>